<commit_message>
Rate check: Bosch model clarifications no longer counted as brand changes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4c5Y1XBRj63SkdBZ73bUS
</commit_message>
<xml_diff>
--- a/quotes/PR-217-228/Quote_PR217_PR228_Rate_Check.xlsx
+++ b/quotes/PR-217-228/Quote_PR217_PR228_Rate_Check.xlsx
@@ -342,7 +342,7 @@
     <t xml:space="preserve">Bosch Professional</t>
   </si>
   <si>
-    <t xml:space="preserve">Bosch GDX 180-Li</t>
+    <t xml:space="preserve">Bosch Professional GDX 180-Li</t>
   </si>
   <si>
     <t xml:space="preserve">ktools 45,000 solo / 79,000 kit; kamadi 75,200</t>
@@ -354,7 +354,7 @@
     <t xml:space="preserve">CORDLESS IMPACT WRENCH 350N (Bosch)</t>
   </si>
   <si>
-    <t xml:space="preserve">Bosch GDS 18V-350</t>
+    <t xml:space="preserve">Bosch Professional GDS 18V-350</t>
   </si>
   <si>
     <t xml:space="preserve">No PK listing; est from GDX/GDS range</t>
@@ -363,7 +363,7 @@
     <t xml:space="preserve">CORDLESS IMPACT WRENCH 1000N (Bosch)</t>
   </si>
   <si>
-    <t xml:space="preserve">Bosch GDS 18V-1000</t>
+    <t xml:space="preserve">Bosch Professional GDS 18V-1000</t>
   </si>
   <si>
     <t xml:space="preserve">ktools 70,000 solo (oos); kamadi 143,800 kit</t>
@@ -426,7 +426,7 @@
     <t xml:space="preserve">DRILL MACHINE CORDLESS ROTARY HAMMER Bosch</t>
   </si>
   <si>
-    <t xml:space="preserve">Bosch GBH 180-LI / GBH 18V-26</t>
+    <t xml:space="preserve">Bosch Professional GBH 180-LI / GBH 18V-26</t>
   </si>
   <si>
     <t xml:space="preserve">ktools 49,000 solo / 115,000 kit</t>
@@ -615,7 +615,7 @@
     <t xml:space="preserve">CORDLESS DRILL DRIVER 150NM Bosch</t>
   </si>
   <si>
-    <t xml:space="preserve">Bosch GSR/GSB 18V-150 C</t>
+    <t xml:space="preserve">Bosch Professional GSR/GSB 18V-150 C</t>
   </si>
   <si>
     <t xml:space="preserve">ktools GSB 18V-150C 199,500 (oos)</t>
@@ -1128,7 +1128,7 @@
     <t xml:space="preserve">CORDLESS SMALL ANGLE GRINDER 125MM EQUIVAL</t>
   </si>
   <si>
-    <t xml:space="preserve">Bosch GWS 180-LI / GWS 18V-10</t>
+    <t xml:space="preserve">Bosch Professional GWS 180-LI / GWS 18V-10</t>
   </si>
   <si>
     <t xml:space="preserve">powerhouseexpress 38,340 solo; ktools 40,000 solo</t>
@@ -1167,7 +1167,7 @@
     <t xml:space="preserve">ANGLE GRINDER 9" BOSCH PRO STONE BONDED CU</t>
   </si>
   <si>
-    <t xml:space="preserve">Bosch GWS 2200-230 H</t>
+    <t xml:space="preserve">Bosch Professional GWS 2200-230 H</t>
   </si>
   <si>
     <t xml:space="preserve">imartpk 36,570; kamadi 43,200; ktools 44,000</t>
@@ -4479,7 +4479,7 @@
       </c>
       <c r="O44" s="6" t="str">
         <f aca="false">IF(ISNUMBER(SEARCH(C44,F44)),"","YES")</f>
-        <v>YES</v>
+        <v/>
       </c>
       <c r="P44" s="6" t="s">
         <v>55</v>
@@ -4542,7 +4542,7 @@
       </c>
       <c r="O45" s="6" t="str">
         <f aca="false">IF(ISNUMBER(SEARCH(C45,F45)),"","YES")</f>
-        <v>YES</v>
+        <v/>
       </c>
       <c r="P45" s="6" t="s">
         <v>24</v>
@@ -4552,7 +4552,7 @@
       </c>
       <c r="R45" s="7"/>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="n">
         <v>42</v>
       </c>
@@ -4603,7 +4603,7 @@
       </c>
       <c r="O46" s="6" t="str">
         <f aca="false">IF(ISNUMBER(SEARCH(C46,F46)),"","YES")</f>
-        <v>YES</v>
+        <v/>
       </c>
       <c r="P46" s="6" t="s">
         <v>55</v>
@@ -5276,7 +5276,7 @@
       </c>
       <c r="O57" s="6" t="str">
         <f aca="false">IF(ISNUMBER(SEARCH(C57,F57)),"","YES")</f>
-        <v>YES</v>
+        <v/>
       </c>
       <c r="P57" s="6" t="s">
         <v>55</v>
@@ -7738,7 +7738,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="6" t="n">
         <v>97</v>
       </c>
@@ -7789,7 +7789,7 @@
       </c>
       <c r="O98" s="6" t="str">
         <f aca="false">IF(ISNUMBER(SEARCH(C98,F98)),"","YES")</f>
-        <v>YES</v>
+        <v/>
       </c>
       <c r="P98" s="6" t="s">
         <v>44</v>
@@ -15255,7 +15255,7 @@
       </c>
       <c r="O220" s="6" t="str">
         <f aca="false">IF(ISNUMBER(SEARCH(C220,F220)),"","YES")</f>
-        <v>YES</v>
+        <v/>
       </c>
       <c r="P220" s="6" t="s">
         <v>55</v>
@@ -15627,7 +15627,7 @@
       </c>
       <c r="O226" s="6" t="str">
         <f aca="false">IF(ISNUMBER(SEARCH(C226,F226)),"","YES")</f>
-        <v>YES</v>
+        <v/>
       </c>
       <c r="P226" s="6" t="s">
         <v>55</v>
@@ -15817,7 +15817,7 @@
       </c>
       <c r="B8" s="11" t="n">
         <f aca="false">COUNTIF('Rate Check'!O6:O227,"YES")</f>
-        <v>127</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
More Pakistani listings: toilet brush, cotton waste, stainless rods
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4c5Y1XBRj63SkdBZ73bUS
</commit_message>
<xml_diff>
--- a/quotes/PR-217-228/Quote_PR217_PR228_Rate_Check.xlsx
+++ b/quotes/PR-217-228/Quote_PR217_PR228_Rate_Check.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1358" uniqueCount="518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1357" uniqueCount="520">
   <si>
     <t xml:space="preserve">Zidane Corporation - Quote PR-217 &amp; PR-228: Brand + Buying Rate Check</t>
   </si>
@@ -1005,10 +1005,16 @@
     <t xml:space="preserve">TOILET CLEANING BRUSH</t>
   </si>
   <si>
+    <t xml:space="preserve">Local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">alclean.pk round toilet brush Rs 203; mjstraders 8142 toilet brush Rs 203</t>
+  </si>
+  <si>
     <t xml:space="preserve">CUT PIECES OF CLOTHS FOR CLEANING</t>
   </si>
   <si>
-    <t xml:space="preserve">Market (per kg)</t>
+    <t xml:space="preserve">nasirnsons.com cotton waste per kg Rs 160 (cleaning cloth/rags)</t>
   </si>
   <si>
     <t xml:space="preserve">ANCHOR BOLT 10X110</t>
@@ -1056,16 +1062,16 @@
     <t xml:space="preserve">SS WELDING RODS 309L-16 2.6MM NO.12</t>
   </si>
   <si>
-    <t xml:space="preserve">Market (pack)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Online nahi mila - dealer quote chahiye. SS 309L</t>
+    <t xml:space="preserve">Stainarc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">priceinfo.pk Stainarc stainless rod 4.0mm 1kg packet Rs 4,200-4,400 (309L 2.6mm exact nahi)</t>
   </si>
   <si>
     <t xml:space="preserve">SS WELDING RODS 316L-16 2.6MM NO.12</t>
   </si>
   <si>
-    <t xml:space="preserve">Online nahi mila - dealer quote chahiye. SS 316L</t>
+    <t xml:space="preserve">priceinfo.pk Stainarc stainless rod 4.0mm 1kg packet Rs 4,200-4,400 (316L 2.6mm exact nahi)</t>
   </si>
   <si>
     <t xml:space="preserve">BLIND RIVETS 04MMX25MM (1000PCS)</t>
@@ -11661,7 +11667,7 @@
       </c>
       <c r="R156" s="7"/>
     </row>
-    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="157" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="6" t="n">
         <v>158</v>
       </c>
@@ -11678,17 +11684,17 @@
         <v>311</v>
       </c>
       <c r="F157" s="7" t="s">
-        <v>297</v>
+        <v>326</v>
       </c>
       <c r="G157" s="9" t="n">
-        <v>150</v>
+        <v>203</v>
       </c>
       <c r="H157" s="9" t="n">
-        <v>250</v>
+        <v>203</v>
       </c>
       <c r="I157" s="10" t="n">
         <f aca="false">IF(E157=0,0,(E157-H157)/E157)</f>
-        <v>0.196141479099678</v>
+        <v>0.347266881028939</v>
       </c>
       <c r="J157" s="6" t="str">
         <f aca="false">IF(E157&lt;G157,"LOSS",IF(E157&lt;H157*1.1,"THIN / RISK",IF(E157&gt;H157*1.8,"OVERPRICED?","OK")))</f>
@@ -11708,28 +11714,26 @@
       </c>
       <c r="N157" s="8" t="n">
         <f aca="false">D157*H157</f>
-        <v>3000</v>
+        <v>2436</v>
       </c>
       <c r="O157" s="6" t="str">
         <f aca="false">IF(ISNUMBER(SEARCH(C157,F157)),"","YES")</f>
         <v>YES</v>
       </c>
       <c r="P157" s="6" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="Q157" s="7" t="s">
-        <v>145</v>
-      </c>
-      <c r="R157" s="7" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>327</v>
+      </c>
+      <c r="R157" s="7"/>
+    </row>
+    <row r="158" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="6" t="n">
         <v>159</v>
       </c>
       <c r="B158" s="7" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C158" s="6" t="s">
         <v>28</v>
@@ -11741,25 +11745,25 @@
         <v>325</v>
       </c>
       <c r="F158" s="7" t="s">
-        <v>297</v>
+        <v>326</v>
       </c>
       <c r="G158" s="9" t="n">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="H158" s="9" t="n">
-        <v>280</v>
+        <v>160</v>
       </c>
       <c r="I158" s="10" t="n">
         <f aca="false">IF(E158=0,0,(E158-H158)/E158)</f>
-        <v>0.138461538461538</v>
+        <v>0.507692307692308</v>
       </c>
       <c r="J158" s="6" t="str">
         <f aca="false">IF(E158&lt;G158,"LOSS",IF(E158&lt;H158*1.1,"THIN / RISK",IF(E158&gt;H158*1.8,"OVERPRICED?","OK")))</f>
-        <v>OK</v>
+        <v>OVERPRICED?</v>
       </c>
       <c r="K158" s="8" t="n">
         <f aca="false">IF(J158="OVERPRICED?",ROUND(H158*1.35,-1),MAX(E158,ROUND(H158*(1+$E$3),-1)))</f>
-        <v>325</v>
+        <v>220</v>
       </c>
       <c r="L158" s="8" t="n">
         <f aca="false">D158*E158</f>
@@ -11767,24 +11771,24 @@
       </c>
       <c r="M158" s="8" t="n">
         <f aca="false">D158*K158</f>
-        <v>32500</v>
+        <v>22000</v>
       </c>
       <c r="N158" s="8" t="n">
         <f aca="false">D158*H158</f>
-        <v>28000</v>
+        <v>16000</v>
       </c>
       <c r="O158" s="6" t="str">
         <f aca="false">IF(ISNUMBER(SEARCH(C158,F158)),"","YES")</f>
         <v>YES</v>
       </c>
       <c r="P158" s="6" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="Q158" s="7" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="R158" s="7" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11792,7 +11796,7 @@
         <v>160</v>
       </c>
       <c r="B159" s="7" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C159" s="6" t="s">
         <v>28</v>
@@ -11804,7 +11808,7 @@
         <v>117</v>
       </c>
       <c r="F159" s="7" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="G159" s="9" t="n">
         <v>65</v>
@@ -11844,7 +11848,7 @@
         <v>24</v>
       </c>
       <c r="Q159" s="7" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="R159" s="7" t="s">
         <v>26</v>
@@ -11855,7 +11859,7 @@
         <v>161</v>
       </c>
       <c r="B160" s="7" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="C160" s="6" t="s">
         <v>28</v>
@@ -11867,7 +11871,7 @@
         <v>169</v>
       </c>
       <c r="F160" s="7" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G160" s="9" t="n">
         <v>90</v>
@@ -11918,7 +11922,7 @@
         <v>162</v>
       </c>
       <c r="B161" s="7" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C161" s="6" t="s">
         <v>28</v>
@@ -11930,7 +11934,7 @@
         <v>234</v>
       </c>
       <c r="F161" s="7" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G161" s="9" t="n">
         <v>120</v>
@@ -11981,7 +11985,7 @@
         <v>164</v>
       </c>
       <c r="B162" s="7" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="C162" s="6" t="s">
         <v>22</v>
@@ -11993,7 +11997,7 @@
         <v>1209</v>
       </c>
       <c r="F162" s="7" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="G162" s="9" t="n">
         <v>1450</v>
@@ -12033,7 +12037,7 @@
         <v>24</v>
       </c>
       <c r="Q162" s="7" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="R162" s="7" t="s">
         <v>26</v>
@@ -12044,7 +12048,7 @@
         <v>165</v>
       </c>
       <c r="B163" s="7" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C163" s="6" t="s">
         <v>22</v>
@@ -12056,7 +12060,7 @@
         <v>1209</v>
       </c>
       <c r="F163" s="7" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="G163" s="9" t="n">
         <v>2248</v>
@@ -12096,7 +12100,7 @@
         <v>24</v>
       </c>
       <c r="Q163" s="7" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="R163" s="7" t="s">
         <v>26</v>
@@ -12107,7 +12111,7 @@
         <v>166</v>
       </c>
       <c r="B164" s="7" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="C164" s="6" t="s">
         <v>22</v>
@@ -12119,7 +12123,7 @@
         <v>3022</v>
       </c>
       <c r="F164" s="7" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="G164" s="9" t="n">
         <v>2325</v>
@@ -12159,7 +12163,7 @@
         <v>24</v>
       </c>
       <c r="Q164" s="7" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="R164" s="7" t="s">
         <v>26</v>
@@ -12170,7 +12174,7 @@
         <v>167</v>
       </c>
       <c r="B165" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C165" s="6" t="s">
         <v>22</v>
@@ -12182,25 +12186,25 @@
         <v>6240</v>
       </c>
       <c r="F165" s="7" t="s">
-        <v>22</v>
+        <v>345</v>
       </c>
       <c r="G165" s="9" t="n">
-        <v>4500</v>
+        <v>4400</v>
       </c>
       <c r="H165" s="9" t="n">
-        <v>6000</v>
+        <v>4400</v>
       </c>
       <c r="I165" s="10" t="n">
         <f aca="false">IF(E165=0,0,(E165-H165)/E165)</f>
-        <v>0.0384615384615385</v>
+        <v>0.294871794871795</v>
       </c>
       <c r="J165" s="6" t="str">
         <f aca="false">IF(E165&lt;G165,"LOSS",IF(E165&lt;H165*1.1,"THIN / RISK",IF(E165&gt;H165*1.8,"OVERPRICED?","OK")))</f>
-        <v>THIN / RISK</v>
+        <v>OK</v>
       </c>
       <c r="K165" s="8" t="n">
         <f aca="false">IF(J165="OVERPRICED?",ROUND(H165*1.35,-1),MAX(E165,ROUND(H165*(1+$E$3),-1)))</f>
-        <v>6900</v>
+        <v>6240</v>
       </c>
       <c r="L165" s="8" t="n">
         <f aca="false">D165*E165</f>
@@ -12208,24 +12212,24 @@
       </c>
       <c r="M165" s="8" t="n">
         <f aca="false">D165*K165</f>
-        <v>276000</v>
+        <v>249600</v>
       </c>
       <c r="N165" s="8" t="n">
         <f aca="false">D165*H165</f>
-        <v>240000</v>
+        <v>176000</v>
       </c>
       <c r="O165" s="6" t="str">
         <f aca="false">IF(ISNUMBER(SEARCH(C165,F165)),"","YES")</f>
-        <v/>
+        <v>YES</v>
       </c>
       <c r="P165" s="6" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="Q165" s="7" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="R165" s="7" t="s">
-        <v>344</v>
+        <v>26</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12233,7 +12237,7 @@
         <v>168</v>
       </c>
       <c r="B166" s="7" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="C166" s="6" t="s">
         <v>22</v>
@@ -12245,25 +12249,25 @@
         <v>7150</v>
       </c>
       <c r="F166" s="7" t="s">
-        <v>22</v>
+        <v>345</v>
       </c>
       <c r="G166" s="9" t="n">
-        <v>5200</v>
+        <v>4400</v>
       </c>
       <c r="H166" s="9" t="n">
-        <v>6800</v>
+        <v>4400</v>
       </c>
       <c r="I166" s="10" t="n">
         <f aca="false">IF(E166=0,0,(E166-H166)/E166)</f>
-        <v>0.048951048951049</v>
+        <v>0.384615384615385</v>
       </c>
       <c r="J166" s="6" t="str">
         <f aca="false">IF(E166&lt;G166,"LOSS",IF(E166&lt;H166*1.1,"THIN / RISK",IF(E166&gt;H166*1.8,"OVERPRICED?","OK")))</f>
-        <v>THIN / RISK</v>
+        <v>OK</v>
       </c>
       <c r="K166" s="8" t="n">
         <f aca="false">IF(J166="OVERPRICED?",ROUND(H166*1.35,-1),MAX(E166,ROUND(H166*(1+$E$3),-1)))</f>
-        <v>7820</v>
+        <v>7150</v>
       </c>
       <c r="L166" s="8" t="n">
         <f aca="false">D166*E166</f>
@@ -12271,24 +12275,24 @@
       </c>
       <c r="M166" s="8" t="n">
         <f aca="false">D166*K166</f>
-        <v>156400</v>
+        <v>143000</v>
       </c>
       <c r="N166" s="8" t="n">
         <f aca="false">D166*H166</f>
-        <v>136000</v>
+        <v>88000</v>
       </c>
       <c r="O166" s="6" t="str">
         <f aca="false">IF(ISNUMBER(SEARCH(C166,F166)),"","YES")</f>
-        <v/>
+        <v>YES</v>
       </c>
       <c r="P166" s="6" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="Q166" s="7" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="R166" s="7" t="s">
-        <v>346</v>
+        <v>26</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12296,7 +12300,7 @@
         <v>177</v>
       </c>
       <c r="B167" s="7" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="C167" s="6" t="s">
         <v>28</v>
@@ -12348,7 +12352,7 @@
         <v>24</v>
       </c>
       <c r="Q167" s="7" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="R167" s="7" t="s">
         <v>26</v>
@@ -12359,7 +12363,7 @@
         <v>179</v>
       </c>
       <c r="B168" s="7" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="C168" s="6" t="s">
         <v>28</v>
@@ -12422,7 +12426,7 @@
         <v>180</v>
       </c>
       <c r="B169" s="7" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="C169" s="6" t="s">
         <v>28</v>
@@ -12485,7 +12489,7 @@
         <v>181</v>
       </c>
       <c r="B170" s="7" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="C170" s="6" t="s">
         <v>28</v>
@@ -12548,7 +12552,7 @@
         <v>182</v>
       </c>
       <c r="B171" s="7" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="C171" s="6" t="s">
         <v>28</v>
@@ -12611,7 +12615,7 @@
         <v>183</v>
       </c>
       <c r="B172" s="7" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="C172" s="6" t="s">
         <v>28</v>
@@ -12674,7 +12678,7 @@
         <v>184</v>
       </c>
       <c r="B173" s="7" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C173" s="6" t="s">
         <v>28</v>
@@ -12737,7 +12741,7 @@
         <v>185</v>
       </c>
       <c r="B174" s="7" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="C174" s="6" t="s">
         <v>28</v>
@@ -12800,7 +12804,7 @@
         <v>186</v>
       </c>
       <c r="B175" s="7" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="C175" s="6" t="s">
         <v>28</v>
@@ -12863,7 +12867,7 @@
         <v>187</v>
       </c>
       <c r="B176" s="7" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="C176" s="6" t="s">
         <v>28</v>
@@ -12926,7 +12930,7 @@
         <v>188</v>
       </c>
       <c r="B177" s="7" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="C177" s="6" t="s">
         <v>28</v>
@@ -12989,7 +12993,7 @@
         <v>189</v>
       </c>
       <c r="B178" s="7" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="C178" s="6" t="s">
         <v>28</v>
@@ -13052,7 +13056,7 @@
         <v>190</v>
       </c>
       <c r="B179" s="7" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="C179" s="6" t="s">
         <v>28</v>
@@ -13115,7 +13119,7 @@
         <v>191</v>
       </c>
       <c r="B180" s="7" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="C180" s="6" t="s">
         <v>28</v>
@@ -13178,7 +13182,7 @@
         <v>192</v>
       </c>
       <c r="B181" s="7" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="C181" s="6" t="s">
         <v>28</v>
@@ -13241,7 +13245,7 @@
         <v>193</v>
       </c>
       <c r="B182" s="7" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="C182" s="6" t="s">
         <v>28</v>
@@ -13304,7 +13308,7 @@
         <v>194</v>
       </c>
       <c r="B183" s="7" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C183" s="6" t="s">
         <v>28</v>
@@ -13367,7 +13371,7 @@
         <v>195</v>
       </c>
       <c r="B184" s="7" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="C184" s="6" t="s">
         <v>28</v>
@@ -13430,7 +13434,7 @@
         <v>196</v>
       </c>
       <c r="B185" s="7" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="C185" s="6" t="s">
         <v>28</v>
@@ -13493,7 +13497,7 @@
         <v>197</v>
       </c>
       <c r="B186" s="7" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="C186" s="6" t="s">
         <v>28</v>
@@ -13545,7 +13549,7 @@
         <v>44</v>
       </c>
       <c r="Q186" s="7" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="R186" s="7"/>
     </row>
@@ -13554,7 +13558,7 @@
         <v>198</v>
       </c>
       <c r="B187" s="7" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C187" s="6" t="s">
         <v>28</v>
@@ -13606,7 +13610,7 @@
         <v>44</v>
       </c>
       <c r="Q187" s="7" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="R187" s="7"/>
     </row>
@@ -13615,7 +13619,7 @@
         <v>199</v>
       </c>
       <c r="B188" s="7" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="C188" s="6" t="s">
         <v>28</v>
@@ -13667,7 +13671,7 @@
         <v>44</v>
       </c>
       <c r="Q188" s="7" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="R188" s="7"/>
     </row>
@@ -13676,7 +13680,7 @@
         <v>200</v>
       </c>
       <c r="B189" s="7" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="C189" s="6" t="s">
         <v>28</v>
@@ -13728,7 +13732,7 @@
         <v>44</v>
       </c>
       <c r="Q189" s="7" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="R189" s="7"/>
     </row>
@@ -13737,7 +13741,7 @@
         <v>201</v>
       </c>
       <c r="B190" s="7" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="C190" s="6" t="s">
         <v>28</v>
@@ -13789,7 +13793,7 @@
         <v>44</v>
       </c>
       <c r="Q190" s="7" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="R190" s="7"/>
     </row>
@@ -13798,7 +13802,7 @@
         <v>202</v>
       </c>
       <c r="B191" s="7" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="C191" s="6" t="s">
         <v>28</v>
@@ -13850,7 +13854,7 @@
         <v>24</v>
       </c>
       <c r="Q191" s="7" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="R191" s="7" t="s">
         <v>26</v>
@@ -13861,7 +13865,7 @@
         <v>204</v>
       </c>
       <c r="B192" s="7" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="C192" s="6" t="s">
         <v>28</v>
@@ -13873,7 +13877,7 @@
         <v>845</v>
       </c>
       <c r="F192" s="7" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="G192" s="9" t="n">
         <v>5480</v>
@@ -13913,7 +13917,7 @@
         <v>30</v>
       </c>
       <c r="Q192" s="7" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="R192" s="7" t="s">
         <v>32</v>
@@ -13924,7 +13928,7 @@
         <v>205</v>
       </c>
       <c r="B193" s="7" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="C193" s="6" t="s">
         <v>28</v>
@@ -13936,7 +13940,7 @@
         <v>910</v>
       </c>
       <c r="F193" s="7" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="G193" s="9" t="n">
         <v>5960</v>
@@ -13976,7 +13980,7 @@
         <v>30</v>
       </c>
       <c r="Q193" s="7" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="R193" s="7" t="s">
         <v>32</v>
@@ -13987,7 +13991,7 @@
         <v>206</v>
       </c>
       <c r="B194" s="7" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="C194" s="6" t="s">
         <v>28</v>
@@ -13999,7 +14003,7 @@
         <v>1170</v>
       </c>
       <c r="F194" s="7" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="G194" s="9" t="n">
         <v>6930</v>
@@ -14039,7 +14043,7 @@
         <v>30</v>
       </c>
       <c r="Q194" s="7" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="R194" s="7" t="s">
         <v>32</v>
@@ -14050,7 +14054,7 @@
         <v>207</v>
       </c>
       <c r="B195" s="7" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="C195" s="6" t="s">
         <v>28</v>
@@ -14062,7 +14066,7 @@
         <v>1430</v>
       </c>
       <c r="F195" s="7" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="G195" s="9" t="n">
         <v>8960</v>
@@ -14102,7 +14106,7 @@
         <v>30</v>
       </c>
       <c r="Q195" s="7" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="R195" s="7" t="s">
         <v>32</v>
@@ -14113,7 +14117,7 @@
         <v>208</v>
       </c>
       <c r="B196" s="7" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="C196" s="6" t="s">
         <v>28</v>
@@ -14125,7 +14129,7 @@
         <v>1690</v>
       </c>
       <c r="F196" s="7" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="G196" s="9" t="n">
         <v>2900</v>
@@ -14165,7 +14169,7 @@
         <v>44</v>
       </c>
       <c r="Q196" s="7" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="R196" s="7"/>
     </row>
@@ -14174,7 +14178,7 @@
         <v>209</v>
       </c>
       <c r="B197" s="7" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="C197" s="6" t="s">
         <v>28</v>
@@ -14186,7 +14190,7 @@
         <v>2340</v>
       </c>
       <c r="F197" s="7" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="G197" s="9" t="n">
         <v>15380</v>
@@ -14226,7 +14230,7 @@
         <v>30</v>
       </c>
       <c r="Q197" s="7" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="R197" s="7" t="s">
         <v>32</v>
@@ -14237,7 +14241,7 @@
         <v>210</v>
       </c>
       <c r="B198" s="7" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="C198" s="6" t="s">
         <v>28</v>
@@ -14249,7 +14253,7 @@
         <v>2860</v>
       </c>
       <c r="F198" s="7" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="G198" s="9" t="n">
         <v>17610</v>
@@ -14289,7 +14293,7 @@
         <v>30</v>
       </c>
       <c r="Q198" s="7" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="R198" s="7" t="s">
         <v>32</v>
@@ -14300,7 +14304,7 @@
         <v>211</v>
       </c>
       <c r="B199" s="7" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C199" s="6" t="s">
         <v>28</v>
@@ -14312,7 +14316,7 @@
         <v>4160</v>
       </c>
       <c r="F199" s="7" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="G199" s="9" t="n">
         <v>22180</v>
@@ -14352,7 +14356,7 @@
         <v>30</v>
       </c>
       <c r="Q199" s="7" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="R199" s="7" t="s">
         <v>32</v>
@@ -14363,7 +14367,7 @@
         <v>212</v>
       </c>
       <c r="B200" s="7" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="C200" s="6" t="s">
         <v>28</v>
@@ -14375,7 +14379,7 @@
         <v>5460</v>
       </c>
       <c r="F200" s="7" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="G200" s="9" t="n">
         <v>25690</v>
@@ -14415,7 +14419,7 @@
         <v>30</v>
       </c>
       <c r="Q200" s="7" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="R200" s="7" t="s">
         <v>32</v>
@@ -14426,7 +14430,7 @@
         <v>213</v>
       </c>
       <c r="B201" s="7" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="C201" s="6" t="s">
         <v>28</v>
@@ -14489,7 +14493,7 @@
         <v>214</v>
       </c>
       <c r="B202" s="7" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="C202" s="6" t="s">
         <v>28</v>
@@ -14552,7 +14556,7 @@
         <v>215</v>
       </c>
       <c r="B203" s="7" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="C203" s="6" t="s">
         <v>28</v>
@@ -14615,7 +14619,7 @@
         <v>216</v>
       </c>
       <c r="B204" s="7" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="C204" s="6" t="s">
         <v>28</v>
@@ -14678,7 +14682,7 @@
         <v>217</v>
       </c>
       <c r="B205" s="7" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="C205" s="6" t="s">
         <v>28</v>
@@ -14741,7 +14745,7 @@
         <v>218</v>
       </c>
       <c r="B206" s="7" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="C206" s="6" t="s">
         <v>28</v>
@@ -14804,7 +14808,7 @@
         <v>219</v>
       </c>
       <c r="B207" s="7" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="C207" s="6" t="s">
         <v>28</v>
@@ -14867,7 +14871,7 @@
         <v>220</v>
       </c>
       <c r="B208" s="7" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="C208" s="6" t="s">
         <v>28</v>
@@ -14930,7 +14934,7 @@
         <v>221</v>
       </c>
       <c r="B209" s="7" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="C209" s="6" t="s">
         <v>28</v>
@@ -14993,7 +14997,7 @@
         <v>222</v>
       </c>
       <c r="B210" s="7" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="C210" s="6" t="s">
         <v>28</v>
@@ -15005,7 +15009,7 @@
         <v>15600</v>
       </c>
       <c r="F210" s="7" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="G210" s="9" t="n">
         <v>18000</v>
@@ -15056,7 +15060,7 @@
         <v>223</v>
       </c>
       <c r="B211" s="7" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="C211" s="6" t="s">
         <v>28</v>
@@ -15108,7 +15112,7 @@
         <v>44</v>
       </c>
       <c r="Q211" s="7" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="R211" s="7"/>
     </row>
@@ -15117,7 +15121,7 @@
         <v>224</v>
       </c>
       <c r="B212" s="7" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="C212" s="6" t="s">
         <v>28</v>
@@ -15129,7 +15133,7 @@
         <v>54600</v>
       </c>
       <c r="F212" s="7" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="G212" s="9" t="n">
         <v>85000</v>
@@ -15169,10 +15173,10 @@
         <v>30</v>
       </c>
       <c r="Q212" s="7" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="R212" s="7" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15180,7 +15184,7 @@
         <v>225</v>
       </c>
       <c r="B213" s="7" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="C213" s="6" t="s">
         <v>28</v>
@@ -15232,7 +15236,7 @@
         <v>30</v>
       </c>
       <c r="Q213" s="7" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="R213" s="7" t="s">
         <v>32</v>
@@ -15243,7 +15247,7 @@
         <v>226</v>
       </c>
       <c r="B214" s="7" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="C214" s="6" t="s">
         <v>28</v>
@@ -15295,7 +15299,7 @@
         <v>30</v>
       </c>
       <c r="Q214" s="7" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="R214" s="7" t="s">
         <v>32</v>
@@ -15306,7 +15310,7 @@
         <v>227</v>
       </c>
       <c r="B215" s="7" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="C215" s="6" t="s">
         <v>28</v>
@@ -15358,7 +15362,7 @@
         <v>30</v>
       </c>
       <c r="Q215" s="7" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="R215" s="7" t="s">
         <v>32</v>
@@ -15369,7 +15373,7 @@
         <v>228</v>
       </c>
       <c r="B216" s="7" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="C216" s="6" t="s">
         <v>28</v>
@@ -15421,7 +15425,7 @@
         <v>30</v>
       </c>
       <c r="Q216" s="7" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="R216" s="7" t="s">
         <v>32</v>
@@ -15432,7 +15436,7 @@
         <v>229</v>
       </c>
       <c r="B217" s="7" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="C217" s="6" t="s">
         <v>28</v>
@@ -15484,7 +15488,7 @@
         <v>30</v>
       </c>
       <c r="Q217" s="7" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="R217" s="7" t="s">
         <v>32</v>
@@ -15495,7 +15499,7 @@
         <v>230</v>
       </c>
       <c r="B218" s="7" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="C218" s="6" t="s">
         <v>28</v>
@@ -15507,7 +15511,7 @@
         <v>9750</v>
       </c>
       <c r="F218" s="7" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="G218" s="9" t="n">
         <v>5950</v>
@@ -15547,7 +15551,7 @@
         <v>24</v>
       </c>
       <c r="Q218" s="7" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="R218" s="7" t="s">
         <v>26</v>
@@ -15558,7 +15562,7 @@
         <v>231</v>
       </c>
       <c r="B219" s="7" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="C219" s="6" t="s">
         <v>28</v>
@@ -15570,7 +15574,7 @@
         <v>12350</v>
       </c>
       <c r="F219" s="7" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="G219" s="9" t="n">
         <v>5950</v>
@@ -15610,7 +15614,7 @@
         <v>44</v>
       </c>
       <c r="Q219" s="7" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="R219" s="7"/>
     </row>
@@ -15619,7 +15623,7 @@
         <v>233</v>
       </c>
       <c r="B220" s="7" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="C220" s="6" t="s">
         <v>111</v>
@@ -15671,7 +15675,7 @@
         <v>44</v>
       </c>
       <c r="Q220" s="7" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="R220" s="7"/>
     </row>
@@ -15680,7 +15684,7 @@
         <v>234</v>
       </c>
       <c r="B221" s="7" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="C221" s="6" t="s">
         <v>22</v>
@@ -15732,7 +15736,7 @@
         <v>24</v>
       </c>
       <c r="Q221" s="7" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="R221" s="7" t="s">
         <v>26</v>
@@ -15743,7 +15747,7 @@
         <v>235</v>
       </c>
       <c r="B222" s="7" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="C222" s="6" t="s">
         <v>28</v>
@@ -15795,7 +15799,7 @@
         <v>24</v>
       </c>
       <c r="Q222" s="7" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="R222" s="7" t="s">
         <v>26</v>
@@ -15806,7 +15810,7 @@
         <v>236</v>
       </c>
       <c r="B223" s="7" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="C223" s="6" t="s">
         <v>22</v>
@@ -15818,7 +15822,7 @@
         <v>2860</v>
       </c>
       <c r="F223" s="7" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="G223" s="9" t="n">
         <v>2400</v>
@@ -15858,10 +15862,10 @@
         <v>30</v>
       </c>
       <c r="Q223" s="7" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="R223" s="7" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
     <row r="224" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15869,7 +15873,7 @@
         <v>237</v>
       </c>
       <c r="B224" s="7" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="C224" s="6" t="s">
         <v>28</v>
@@ -15921,7 +15925,7 @@
         <v>24</v>
       </c>
       <c r="Q224" s="7" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="R224" s="7" t="s">
         <v>26</v>
@@ -15932,7 +15936,7 @@
         <v>238</v>
       </c>
       <c r="B225" s="7" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="C225" s="6" t="s">
         <v>28</v>
@@ -15944,7 +15948,7 @@
         <v>8450</v>
       </c>
       <c r="F225" s="7" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="G225" s="9" t="n">
         <v>7800</v>
@@ -15984,7 +15988,7 @@
         <v>44</v>
       </c>
       <c r="Q225" s="7" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="R225" s="7"/>
     </row>
@@ -15993,7 +15997,7 @@
         <v>239</v>
       </c>
       <c r="B226" s="7" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="C226" s="6" t="s">
         <v>111</v>
@@ -16045,7 +16049,7 @@
         <v>44</v>
       </c>
       <c r="Q226" s="7" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="R226" s="7"/>
     </row>
@@ -16054,7 +16058,7 @@
         <v>240</v>
       </c>
       <c r="B227" s="7" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="C227" s="6" t="s">
         <v>28</v>
@@ -16106,15 +16110,15 @@
         <v>30</v>
       </c>
       <c r="Q227" s="7" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="R227" s="7" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
     </row>
     <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B228" s="3" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="L228" s="11" t="n">
         <f aca="false">SUM(L6:L227)</f>
@@ -16122,11 +16126,11 @@
       </c>
       <c r="M228" s="11" t="n">
         <f aca="false">SUM(M6:M227)</f>
-        <v>14711711</v>
+        <v>14661411</v>
       </c>
       <c r="N228" s="11" t="n">
         <f aca="false">SUM(N6:N227)</f>
-        <v>11738936</v>
+        <v>11614372</v>
       </c>
     </row>
   </sheetData>
@@ -16175,12 +16179,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="12" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B3" s="11" t="n">
         <f aca="false">COUNTA('Rate Check'!A6:A227)</f>
@@ -16189,7 +16193,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B4" s="11" t="n">
         <f aca="false">COUNTIF('Rate Check'!J6:J227,"LOSS")</f>
@@ -16198,38 +16202,38 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B5" s="11" t="n">
         <f aca="false">COUNTIF('Rate Check'!J6:J227,"THIN / RISK")</f>
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B6" s="11" t="n">
         <f aca="false">COUNTIF('Rate Check'!J6:J227,"OK")</f>
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B7" s="11" t="n">
         <f aca="false">COUNTIF('Rate Check'!J6:J227,"OVERPRICED?")</f>
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B8" s="11" t="n">
         <f aca="false">COUNTIF('Rate Check'!O6:O227,"YES")</f>
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16237,7 +16241,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B10" s="11" t="n">
         <f aca="false">'Rate Check'!L228</f>
@@ -16246,34 +16250,34 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B11" s="11" t="n">
         <f aca="false">'Rate Check'!N228</f>
-        <v>11738936</v>
+        <v>11614372</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B12" s="11" t="n">
         <f aca="false">B10-B11</f>
-        <v>470572</v>
+        <v>595136</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B13" s="14" t="n">
         <f aca="false">IF(B10=0,0,B12/B10)</f>
-        <v>0.0385414383609888</v>
+        <v>0.04874365125933</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B14" s="11" t="n">
         <f aca="false">SUMPRODUCT(('Rate Check'!E6:E227&lt;'Rate Check'!H6:H227)*('Rate Check'!H6:H227-'Rate Check'!E6:E227)*'Rate Check'!D6:D227)</f>
@@ -16285,20 +16289,20 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B16" s="11" t="n">
         <f aca="false">'Rate Check'!M228</f>
-        <v>14711711</v>
+        <v>14661411</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B17" s="14" t="n">
         <f aca="false">IF(B16=0,0,(B16-B11)/B16)</f>
-        <v>0.202068610510361</v>
+        <v>0.207827132054343</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16306,29 +16310,29 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B19" s="11" t="n">
         <f aca="false">COUNTIF('Rate Check'!P6:P227,"V")</f>
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B20" s="11" t="n">
         <f aca="false">COUNTIF('Rate Check'!P6:P227,"S")</f>
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B21" s="11" t="n">
         <f aca="false">COUNTIF('Rate Check'!P6:P227,"N")</f>
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -16356,247 +16360,247 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="13" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
     </row>
   </sheetData>

</xml_diff>